<commit_message>
Update EU steel TRQ data
</commit_message>
<xml_diff>
--- a/public/data/eu-steel-trq-flat-dashboard.xlsx
+++ b/public/data/eu-steel-trq-flat-dashboard.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1A Non Alloy and Other Alloy Ho" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1B Non Alloy and Other Alloy Ho" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Non Alloy and Other Alloy Col" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3A Electrical Sheets (other tha" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3B Electrical Sheets (other tha" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4A Metallic Coated Sheets" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4B Metallic Coated Sheets" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5 Organic Coated Sheets" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6 Tin Mill Products" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7 Non Alloy and Other Alloy Qua" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8 Stainless Hot Rolled Sheets a" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9 Stainless Cold Rolled Sheets " sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Stainless Hot Rolled Quarto " sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="1A Non Alloy and Other Alloy Ho" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="1B Non Alloy and Other Alloy Ho" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2 Non Alloy and Other Alloy Col" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="3A Electrical Sheets (other tha" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="3B Electrical Sheets (other tha" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="4A Metallic Coated Sheets" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="4B Metallic Coated Sheets" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="5 Organic Coated Sheets" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="6 Tin Mill Products" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="7 Non Alloy and Other Alloy Qua" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="8 Stainless Hot Rolled Sheets a" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="9 Stainless Cold Rolled Sheets " sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="10 Stainless Hot Rolled Quarto " sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>